<commit_message>
experiments: add timing benchmark summary
</commit_message>
<xml_diff>
--- a/本地计划表.xlsx
+++ b/本地计划表.xlsx
@@ -668,7 +668,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>已完成第一版：已在 airfogsim_mechanism_report.md 中整理复杂度表达式和谨慎表述；还需要后续补计时实验。</t>
+          <t>已完成第一版：已在 airfogsim_mechanism_report.md 中整理复杂度表达式，并补充 timing_v0 实测计时。当前小场景下 AirFogSim 约 5.96 ms/step，3-step rollout 约 17.88 ms，Ridge 推理约 0.0044 ms/sample。</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>进行中：前三类图已完成，状态转移流程图已完成；还可补一张复杂度对比示意图或计时实验图。</t>
+          <t>已完成第一版：baseline、扰动、置信区间、状态转移、复杂度对比和计时实验图均已完成；后续可根据 PPT 需要继续精简。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
experiments: add multi-seed simulation summary
</commit_message>
<xml_diff>
--- a/本地计划表.xlsx
+++ b/本地计划表.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$1:$D$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>已完成：已在 airfogsim_mechanism_report.md 中列出随机性来源；当前 demo 设置固定 seed，因此本次导出轨迹可复现。</t>
+          <t>已完成：已在 airfogsim_mechanism_report.md 中列出随机性来源，并完成 multiseed_v0。5 个 seed 下最终车辆数 6-13、任务数 11-37、成功率 0.829-0.969，说明同一场景可产生不同随机轨迹。</t>
         </is>
       </c>
     </row>
@@ -724,17 +724,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>补充严格动作变量</t>
+          <t>构造多 seed 数据集</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>如果 baseline、扰动和置信区间完成较快，再继续导出卸载动作、RB/CPU 分配动作和 UAV 移动动作，为动作条件 world model 做准备；本周不是第一优先级。</t>
+          <t>把 multiseed_v0 的多条仿真轨迹进一步整理成 dataset_multiseed_v0，形成跨随机轨迹的历史窗口-未来标签样本，用于验证模型泛化能力和多场景/多 seed 预训练可行性。</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>未开始。</t>
+          <t>未开始：已有 multiseed_v0 原始统计结果，下一步需要导出 node/link/task 明细并统一构造成训练样本。</t>
         </is>
       </c>
     </row>
@@ -746,22 +746,44 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
+          <t>补充严格动作变量</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>如果 baseline、扰动和置信区间完成较快，再继续导出卸载动作、RB/CPU 分配动作和 UAV 移动动作，为动作条件 world model 做准备；本周不是第一优先级。</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>未开始。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
           <t>更新研究进展文档和下周 PPT</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>将 baseline 结果、扰动实验、置信区间和 AirFogSim 机制分析写入研究进展文档；下周 PPT 围绕实验结果和复杂度、随机性、置信区间三点组织。</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>未开始。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D13"/>
+  <autoFilter ref="A1:D14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
experiments: add dataset multiseed v0
</commit_message>
<xml_diff>
--- a/本地计划表.xlsx
+++ b/本地计划表.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$1:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$1:$D$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -734,29 +734,29 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>未开始：已有 multiseed_v0 原始统计结果，下一步需要导出 node/link/task 明细并统一构造成训练样本。</t>
+          <t>已完成：已导出 5 个 seed 的 node/link/task 明细日志，并构造 dataset_multiseed_v0。总样本数 950，每个 seed 190 个样本，张量形状与 dataset_v0 兼容。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="72" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>补充严格动作变量</t>
+          <t>做跨 seed baseline 泛化实验</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>如果 baseline、扰动和置信区间完成较快，再继续导出卸载动作、RB/CPU 分配动作和 UAV 移动动作，为动作条件 world model 做准备；本周不是第一优先级。</t>
+          <t>基于 dataset_multiseed_v0 做 seed 级训练/测试划分，例如 seed 0-3 训练、seed 4 测试。比较单 seed 测试和跨 seed 测试的误差，用于判断当前 baseline 是否只记住单条轨迹。</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>未开始。</t>
+          <t>未开始：dataset_multiseed_v0 已准备好，下一步直接训练和评估。</t>
         </is>
       </c>
     </row>
@@ -768,22 +768,44 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
+          <t>补充严格动作变量</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>如果 baseline、扰动和置信区间完成较快，再继续导出卸载动作、RB/CPU 分配动作和 UAV 移动动作，为动作条件 world model 做准备；本周不是第一优先级。</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>未开始。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
           <t>更新研究进展文档和下周 PPT</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>将 baseline 结果、扰动实验、置信区间和 AirFogSim 机制分析写入研究进展文档；下周 PPT 围绕实验结果和复杂度、随机性、置信区间三点组织。</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>未开始。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D14"/>
+  <autoFilter ref="A1:D15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
experiments: add cross-seed and action proxy summaries
</commit_message>
<xml_diff>
--- a/本地计划表.xlsx
+++ b/本地计划表.xlsx
@@ -83,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -98,6 +98,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -465,13 +468,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="105" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -756,7 +759,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>未开始：dataset_multiseed_v0 已准备好，下一步直接训练和评估。</t>
+          <t>已完成：run_cross_seed_baseline_v0.py 已完成 seed 0/1/2 训练、seed 3 验证、seed 4 测试。测试 seed 4 上 persistence 全部 RMSE=1.530，Ridge residual 全部 RMSE=3.303，说明当前紧凑线性 residual baseline 跨随机轨迹泛化不足，后续需要双图/动作条件 world model。</t>
         </is>
       </c>
     </row>
@@ -778,7 +781,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>未开始。</t>
+          <t>已完成第一版动作代理接口：build_action_proxy_v0.py 从可观测日志中构造 action_proxy_v0，a_hist=(950,8,13)，a_future=(950,3,13)，包含卸载计数、RB 分配代理、CPU 进度代理和 UAV 移动代理。严格调度动作日志尚未完成，下一步需要在 scheduler 执行时直接记录 offload route、RB indices、CPU allocation、UAV mobility command。</t>
         </is>
       </c>
     </row>
@@ -800,7 +803,73 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>未开始。</t>
+          <t>已完成本周结果文档更新：weekly_result_summary_v0.md、README.md、experiments/airfogsim_v0/README.md 和 AGENTS.md 已同步。PPT 可基于当前图表与报告再整理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>严格动作日志导出</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>在 AirFogSim 调度器执行前后直接记录每个时间步的真实动作：任务卸载目标、通信 RB 编号、CPU 分配量、UAV 移动角度/速度/目标点。用于替代当前 action_proxy_v0 的代理变量。</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>未开始：已有 action_proxy_v0 作为过渡版本。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>双图 baseline / world model 雏形</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>基于 dataset_multiseed_v0 和 action_proxy_v0，搭建比 Ridge 更结构化的模型输入：物理图、通信图、任务状态和动作变量。先做可训练 baseline，再逐步升级为动作条件 latent world model。</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>未开始：当前已证明简单 residual baseline 跨 seed 泛化不足。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>扰动训练实验</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>在训练阶段加入输入扰动或数据增强，再与当前 clean 训练/noisy 测试结果对比，判断鲁棒性是否改善。</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>未开始：当前已完成扰动测试流程。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
experiments: add strict action log summary
</commit_message>
<xml_diff>
--- a/本地计划表.xlsx
+++ b/本地计划表.xlsx
@@ -781,7 +781,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>已完成第一版动作代理接口：build_action_proxy_v0.py 从可观测日志中构造 action_proxy_v0，a_hist=(950,8,13)，a_future=(950,3,13)，包含卸载计数、RB 分配代理、CPU 进度代理和 UAV 移动代理。严格调度动作日志尚未完成，下一步需要在 scheduler 执行时直接记录 offload route、RB indices、CPU allocation、UAV mobility command。</t>
+          <t>已完成：先完成 action_proxy_v0，再完成 strict_action_v0。当前优先使用 strict_action_v0，其中 a_hist=(950,8,13)，a_future=(950,3,13)，动作来自 scheduler 直接记录，包括 offload route、RB indices、CPU allocation、UAV mobility command。</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>未开始：已有 action_proxy_v0 作为过渡版本。</t>
+          <t>已完成：export_strict_actions_v0.py 已直接在 AirFogSim scheduler 决策时记录严格动作日志。已记录卸载目标、回传 RSU、RB indices、CPU allocation、UAV mobility command；并构造 strict_action_v0_samples.npz，a_hist=(950,8,13)，a_future=(950,3,13)。每个 seed 的明细 CSV 已保存在 reports/strict_action_v0/seed_*/。</t>
         </is>
       </c>
     </row>

</xml_diff>